<commit_message>
collection of parts in spreadsheet
</commit_message>
<xml_diff>
--- a/schematic-design/Partslist_Group_PE04_2 - With HSRW.xlsx
+++ b/schematic-design/Partslist_Group_PE04_2 - With HSRW.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Projects\pe04\schematic-design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFEBE582-9EB0-4947-90E2-B5CA8B45C980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831B8F7C-A46F-4548-AEF4-EB4814D2FC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-10800" yWindow="6720" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="5" r:id="rId1"/>
@@ -396,9 +396,6 @@
     <t>1N5908</t>
   </si>
   <si>
-    <t>TVS Diode 5V,</t>
-  </si>
-  <si>
     <t>ST</t>
   </si>
   <si>
@@ -415,6 +412,9 @@
   </si>
   <si>
     <t>https://www.mouser.de/ProductDetail/GCT/USB3145-30-1-A?qs=KUoIvG%2F9IlYD1lvSRu5iyg%3D%3D</t>
+  </si>
+  <si>
+    <t>TVS Diode 5V</t>
   </si>
 </sst>
 </file>
@@ -837,45 +837,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -889,6 +850,45 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1215,38 +1215,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="52"/>
+      <c r="B1" s="48"/>
       <c r="C1" s="17" t="s">
         <v>48</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="56" t="s">
+      <c r="H1" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="52"/>
+      <c r="B2" s="48"/>
       <c r="C2" s="18" t="s">
         <v>49</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="57" t="s">
+      <c r="H2" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -1486,19 +1486,19 @@
         <v>1</v>
       </c>
       <c r="C11" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="D11" s="26" t="s">
-        <v>124</v>
-      </c>
       <c r="E11" s="26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F11" s="26" t="s">
         <v>30</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H11" s="34">
         <v>0.66200000000000003</v>
@@ -1508,7 +1508,7 @@
         <v>0.66200000000000003</v>
       </c>
       <c r="J11" s="35" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
@@ -1616,10 +1616,10 @@
         <v>2</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E15" s="26" t="s">
         <v>119</v>
@@ -1631,7 +1631,7 @@
       <c r="H15" s="34"/>
       <c r="I15" s="33"/>
       <c r="J15" s="35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -1999,10 +1999,10 @@
       <c r="J27" s="35"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="G29" s="58" t="s">
+      <c r="G29" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="H29" s="58"/>
+      <c r="H29" s="45"/>
       <c r="I29" s="10">
         <f>SUM(I5:I27)</f>
         <v>22.038999999999998</v>
@@ -2017,10 +2017,10 @@
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
       <c r="E30" s="13"/>
-      <c r="G30" s="59" t="s">
+      <c r="G30" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="H30" s="59"/>
+      <c r="H30" s="46"/>
       <c r="I30" s="8">
         <f>I29*0.19</f>
         <v>4.1874099999999999</v>
@@ -2028,21 +2028,21 @@
       <c r="J30" s="42"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="53" t="s">
+      <c r="A31" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="B31" s="54"/>
+      <c r="B31" s="50"/>
       <c r="C31" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D31" s="54" t="s">
+      <c r="D31" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="E31" s="55"/>
-      <c r="G31" s="59" t="s">
+      <c r="E31" s="53"/>
+      <c r="G31" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="H31" s="59"/>
+      <c r="H31" s="46"/>
       <c r="I31" s="9">
         <f>I29*1.19</f>
         <v>26.226409999999998</v>
@@ -2050,71 +2050,71 @@
       <c r="J31" s="42"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" s="43" t="s">
+      <c r="A32" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="44"/>
+      <c r="B32" s="52"/>
       <c r="C32" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D32" s="47" t="s">
+      <c r="D32" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="E32" s="48"/>
+      <c r="E32" s="57"/>
       <c r="I32" s="41"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="43" t="s">
+      <c r="A33" s="51" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="44"/>
+      <c r="B33" s="52"/>
       <c r="C33" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D33" s="47" t="s">
+      <c r="D33" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="48"/>
+      <c r="E33" s="57"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="43" t="s">
+      <c r="A34" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="44"/>
+      <c r="B34" s="52"/>
       <c r="C34" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="47" t="s">
+      <c r="D34" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="E34" s="48"/>
+      <c r="E34" s="57"/>
       <c r="H34" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="45" t="s">
+      <c r="A35" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="B35" s="46"/>
+      <c r="B35" s="55"/>
       <c r="C35" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D35" s="49" t="s">
+      <c r="D35" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="E35" s="50"/>
+      <c r="E35" s="59"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="45" t="s">
+      <c r="A36" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="B36" s="46"/>
+      <c r="B36" s="55"/>
       <c r="C36" s="16"/>
-      <c r="D36" s="49" t="s">
+      <c r="D36" s="58" t="s">
         <v>33</v>
       </c>
-      <c r="E36" s="50"/>
+      <c r="E36" s="59"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="2"/>
@@ -2214,16 +2214,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D31:E31"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A36:B36"/>
@@ -2233,6 +2223,16 @@
     <mergeCell ref="D36:E36"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="D35:E35"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G31:H31"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="3">

</xml_diff>